<commit_message>
Display case flags and support tabs to the respective users
</commit_message>
<xml_diff>
--- a/ccd-definitions/jurisdictions/england-wales/data/ccd-template.xlsx
+++ b/ccd-definitions/jurisdictions/england-wales/data/ccd-template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
   <workbookPr showInkAnnotation="0" codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tensaybulcha/Documents/GitHub/Reformed-ET/et-ccd-definitions-englandwales/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rajaram/Projects/et-ccd-callbacks/ccd-definitions/jurisdictions/england-wales/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C51F886-9A3C-FB4B-9A59-BA1C8DAD725B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A1D47BA-1D9B-284B-9C37-9CD01188781F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="55340" yWindow="600" windowWidth="35960" windowHeight="17400" tabRatio="500" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17720" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SearchCriteria" sheetId="37" r:id="rId1"/>
@@ -52,7 +52,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">CaseField!$A$3:$L$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="21" hidden="1">CaseRoles!$A$3:$F$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">CaseType!$A$3:$I$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">CaseTypeTab!$A$3:$J$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">CaseTypeTab!$A$3:$K$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">ComplexTypes!$A$3:$P$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'EnglandWales Scrubbed'!$A$3:$D$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">EventToComplexTypes!$A$3:$I$382</definedName>
@@ -83,7 +83,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3741" uniqueCount="1161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3743" uniqueCount="1162">
   <si>
     <t>Jurisdiction</t>
   </si>
@@ -3655,6 +3655,9 @@
   </si>
   <si>
     <t>Magnitude in number of days that a Time to Live(TTL) value is incremented by</t>
+  </si>
+  <si>
+    <t>This will allow you to display the tab based on access profile</t>
   </si>
 </sst>
 </file>
@@ -26654,7 +26657,7 @@
       <c r="I1" s="266"/>
       <c r="J1" s="265"/>
     </row>
-    <row r="2" spans="1:10" ht="409.6">
+    <row r="2" spans="1:10" ht="204">
       <c r="A2" s="263" t="s">
         <v>1133</v>
       </c>
@@ -29997,7 +30000,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <sheetPr codeName="Sheet6"/>
-  <dimension ref="A1:J119"/>
+  <dimension ref="A1:K119"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="13"/>
   <cols>
     <col min="1" max="1" width="17.1640625" customWidth="1"/>
@@ -30013,7 +30016,7 @@
     <col min="11" max="1015" width="8.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="18">
+    <row r="1" spans="1:11" ht="18">
       <c r="A1" s="30" t="s">
         <v>42</v>
       </c>
@@ -30031,7 +30034,7 @@
       <c r="H1" s="31"/>
       <c r="I1" s="31"/>
     </row>
-    <row r="2" spans="1:10" ht="98">
+    <row r="2" spans="1:11" ht="126">
       <c r="A2" s="23" t="s">
         <v>33</v>
       </c>
@@ -30062,8 +30065,11 @@
       <c r="J2" s="22" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" ht="42">
+      <c r="K2" s="22" t="s">
+        <v>1161</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="42">
       <c r="A3" s="35" t="s">
         <v>39</v>
       </c>
@@ -30094,63 +30100,66 @@
       <c r="J3" s="36" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="4" spans="1:10">
+      <c r="K3" s="36" t="s">
+        <v>763</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
       <c r="D4" s="112"/>
       <c r="E4" s="7"/>
       <c r="G4" s="7"/>
       <c r="H4" s="37"/>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:11">
       <c r="E5" s="7"/>
       <c r="G5" s="7"/>
       <c r="H5" s="37"/>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:11">
       <c r="E6" s="7"/>
       <c r="G6" s="7"/>
       <c r="H6" s="37"/>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:11">
       <c r="E7" s="7"/>
       <c r="G7" s="7"/>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:11">
       <c r="E8" s="7"/>
       <c r="G8" s="7"/>
     </row>
-    <row r="9" spans="1:10">
+    <row r="9" spans="1:11">
       <c r="E9" s="7"/>
       <c r="G9" s="7"/>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:11">
       <c r="E10" s="7"/>
       <c r="G10" s="7"/>
       <c r="H10" s="37"/>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:11">
       <c r="E11" s="7"/>
       <c r="G11" s="7"/>
     </row>
-    <row r="12" spans="1:10">
+    <row r="12" spans="1:11">
       <c r="E12" s="7"/>
       <c r="G12" s="7"/>
     </row>
-    <row r="13" spans="1:10">
+    <row r="13" spans="1:11">
       <c r="E13" s="7"/>
       <c r="G13" s="7"/>
     </row>
-    <row r="14" spans="1:10">
+    <row r="14" spans="1:11">
       <c r="E14" s="7"/>
       <c r="G14" s="7"/>
       <c r="H14" s="37"/>
     </row>
-    <row r="15" spans="1:10">
+    <row r="15" spans="1:11">
       <c r="E15" s="7"/>
       <c r="G15" s="7"/>
       <c r="H15" s="37"/>
     </row>
-    <row r="16" spans="1:10">
+    <row r="16" spans="1:11">
       <c r="E16" s="7"/>
       <c r="G16" s="7"/>
     </row>
@@ -30573,7 +30582,10 @@
       <c r="F119" s="105"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:J3" xr:uid="{561AF9F7-DEF4-214D-AC1D-3FA58FDFD9E6}"/>
+  <autoFilter ref="A3:K3" xr:uid="{00000000-0001-0000-0500-000000000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:K3">
+    <sortCondition ref="K3"/>
+  </sortState>
   <phoneticPr fontId="30" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup paperSize="9" firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>